<commit_message>
CD-182: Add missing regular expressions to the "regex_to_formula" worksheet
</commit_message>
<xml_diff>
--- a/images/rembi_image_schema_main_v0.1.xlsx
+++ b/images/rembi_image_schema_main_v0.1.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10322"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10419"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/providen/Documents/EI/Projects/COPO-schemas/images/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5E524238-05E2-804F-9327-1C68B82FD947}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{68545C1D-1E3E-C244-A8C9-079F6154A3C4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="32820" yWindow="620" windowWidth="30240" windowHeight="17920" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="18080" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="data" sheetId="1" r:id="rId1"/>
@@ -47,7 +47,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1167" uniqueCount="518">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1181" uniqueCount="525">
   <si>
     <t>copo_name</t>
   </si>
@@ -1676,6 +1676,27 @@
   </si>
   <si>
     <t>The file name of the image including the extension. Common file names end with tiff, jpeg, png, gif, bmp, and ome-tiff etc.</t>
+  </si>
+  <si>
+    <t>LEN({column_letter}{row_start})&gt;=25</t>
+  </si>
+  <si>
+    <t>{column_letter}{row_start}=1.5</t>
+  </si>
+  <si>
+    <t>AND(LEFT({column_letter}{row_start},3)="10.",ISNUMBER(SEARCH("/",{column_letter}{row_start})),LEN({column_letter}{row_start})&gt;=10)</t>
+  </si>
+  <si>
+    <t>AND(LEN({column_letter}{row_start})=4,VALUE({column_letter}{row_start})&gt;=1900,VALUE({column_letter}{row_start})&lt;=2099)</t>
+  </si>
+  <si>
+    <t>AND(ISNUMBER(VALUE({column_letter}{row_start})),LEN({column_letter}{row_start})&lt;=8)</t>
+  </si>
+  <si>
+    <t>AND(ISNUMBER(VALUE({column_letter}{row_start})),{column_letter}{row_start}&lt;&gt;"")</t>
+  </si>
+  <si>
+    <t>AND(LEN({column_letter}{row_start})=20, MID({column_letter}{row_start},5,1)="-", MID({column_letter}{row_start},8,1)="-", MID({column_letter}{row_start},11,1)="T", RIGHT({column_letter}{row_start},1)="Z")</t>
   </si>
 </sst>
 </file>
@@ -1743,7 +1764,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="34">
+  <borders count="35">
     <border>
       <left/>
       <right/>
@@ -2180,11 +2201,26 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="76">
+  <cellXfs count="78">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -2407,6 +2443,12 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="34" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="34" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -9724,7 +9766,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:C58"/>
+  <dimension ref="A1:C65"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="41.5" style="15" bestFit="1" customWidth="1"/>
@@ -10300,13 +10342,76 @@
       <c r="C57" s="14"/>
     </row>
     <row r="58" spans="1:3" s="8" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A58" s="10" t="s">
+      <c r="A58" s="13" t="s">
         <v>149</v>
       </c>
-      <c r="B58" s="10" t="s">
+      <c r="B58" s="13" t="s">
         <v>150</v>
       </c>
-      <c r="C58" s="11"/>
+      <c r="C58" s="14"/>
+    </row>
+    <row r="59" spans="1:3" ht="16" x14ac:dyDescent="0.2">
+      <c r="A59" s="76" t="s">
+        <v>223</v>
+      </c>
+      <c r="B59" s="76" t="s">
+        <v>518</v>
+      </c>
+      <c r="C59" s="77"/>
+    </row>
+    <row r="60" spans="1:3" ht="16" x14ac:dyDescent="0.2">
+      <c r="A60" s="76" t="s">
+        <v>247</v>
+      </c>
+      <c r="B60" s="76" t="s">
+        <v>519</v>
+      </c>
+      <c r="C60" s="77"/>
+    </row>
+    <row r="61" spans="1:3" ht="32" x14ac:dyDescent="0.2">
+      <c r="A61" s="76" t="s">
+        <v>266</v>
+      </c>
+      <c r="B61" s="76" t="s">
+        <v>520</v>
+      </c>
+      <c r="C61" s="77"/>
+    </row>
+    <row r="62" spans="1:3" ht="32" x14ac:dyDescent="0.2">
+      <c r="A62" s="76" t="s">
+        <v>270</v>
+      </c>
+      <c r="B62" s="76" t="s">
+        <v>521</v>
+      </c>
+      <c r="C62" s="77"/>
+    </row>
+    <row r="63" spans="1:3" ht="16" x14ac:dyDescent="0.2">
+      <c r="A63" s="76" t="s">
+        <v>275</v>
+      </c>
+      <c r="B63" s="76" t="s">
+        <v>522</v>
+      </c>
+      <c r="C63" s="77"/>
+    </row>
+    <row r="64" spans="1:3" ht="16" x14ac:dyDescent="0.2">
+      <c r="A64" s="76" t="s">
+        <v>361</v>
+      </c>
+      <c r="B64" s="76" t="s">
+        <v>523</v>
+      </c>
+      <c r="C64" s="77"/>
+    </row>
+    <row r="65" spans="1:3" ht="24" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A65" s="76" t="s">
+        <v>437</v>
+      </c>
+      <c r="B65" s="76" t="s">
+        <v>524</v>
+      </c>
+      <c r="C65" s="77"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>